<commit_message>
docs(validation): catch the validation workbooks up with this cycle
- Diag: move the item-6 defect record out of برنامه تست into ثبت ایراد
  (it was appended to the wrong sheet in dbd1bb0); test row 13 stays.
- EspLink EL-020 (new): panel hard-block of green min-off > period
  (8efddaa); host logic verified in 6 cases, live panel/board pending.
- Rtos RT-011 (new, both copies of Rtos_Validation.xlsx kept in sync):
  IWDG check-ins take ms via rtos_time.h (004fbf1); board pending.
  Rtos README test line now says RT-001..RT-011.
- Charger CH-039 (new): charger suspension around flash saves; the
  Diag periodic save joined the NVM/CalLut triggers in 2da0ed1;
  board pending.

All other workbooks audited: no code change this cycle, statuses are
within the allowed set (در انتظار/قبول/رد/مسدود/نیاز به تکرار); their
pending rows are real board tests and were left untouched. Both gates
green.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Charger/Charger_Validation.xlsx
+++ b/Firmware/Modules/Charger/Charger_Validation.xlsx
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2203,14 +2203,11 @@
           <t>نیاز به تکرار</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr">
         <is>
           <t>thermal</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -2273,14 +2270,11 @@
           <t>نیاز به تکرار</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr">
         <is>
           <t>thermal</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -2343,7 +2337,6 @@
           <t>قبول</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
           <t>کد بازبینی</t>
@@ -2354,10 +2347,81 @@
           <t>thermal</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr">
         <is>
           <t>2026-10-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CH-039</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>تعلیق شارژر هنگام ذخیرهٔ فلش</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>بالا</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>شارژ فعال (BULK)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>حین شارژ صبر کن تا یک ذخیرهٔ فلش رخ دهد (ذخیرهٔ NVM یا CalLut از پنل، یا ذخیرهٔ دوره‌ای Diag حدود هر ۶۰ ثانیه) و گیت‌های PWM هر دو کانال را با اسکوپ ببین</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>شارژ فعال + ذخیرهٔ فلش</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2s</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>دور پاک/نوشتن فلش هر دو گیت PWM متوقف و خروجی صفر شود؛ بلافاصله بعد از ذخیره شارژ بدون پرش ادامه یابد</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>هیچ پالس PWM حین پاک‌کردن صفحه دیده نشود و رکورد/تنظیم سالم ذخیره شود</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>هاست 2026-10-15: هر دو گیت سبز (مسیر Diag با 2da0ed1 اضافه شد، NVM/CalLut از قبل بود)؛ تست برد: در انتظار</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>در انتظار</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>2da0ed1</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>

</xml_diff>